<commit_message>
results with larger memory
</commit_message>
<xml_diff>
--- a/benchmarking/results-dist-scaling123.xlsx
+++ b/benchmarking/results-dist-scaling123.xlsx
@@ -1395,7 +1395,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="1">
-        <v>15006</v>
+        <v>30002</v>
       </c>
       <c r="G3" s="1">
         <v>1</v>
@@ -1404,7 +1404,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="1">
-        <v>161.105</v>
+        <v>297.304</v>
       </c>
       <c r="J3" s="1">
         <v>3000</v>
@@ -1631,7 +1631,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="1">
-        <v>15006</v>
+        <v>30009</v>
       </c>
       <c r="G4" s="1">
         <v>1</v>
@@ -1640,7 +1640,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="1">
-        <v>161.705</v>
+        <v>299.488</v>
       </c>
       <c r="J4" s="1">
         <v>3000</v>
@@ -1867,7 +1867,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="1">
-        <v>15008</v>
+        <v>30001</v>
       </c>
       <c r="G5" s="1">
         <v>1</v>
@@ -1876,7 +1876,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="1">
-        <v>162.406</v>
+        <v>296.705</v>
       </c>
       <c r="J5" s="1">
         <v>3000</v>
@@ -2103,7 +2103,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="1">
-        <v>15012</v>
+        <v>30005</v>
       </c>
       <c r="G6" s="1">
         <v>1</v>
@@ -2112,7 +2112,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="1">
-        <v>161.305</v>
+        <v>298.005</v>
       </c>
       <c r="J6" s="1">
         <v>3000</v>
@@ -2339,7 +2339,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="1">
-        <v>15005</v>
+        <v>30002</v>
       </c>
       <c r="G7" s="1">
         <v>1</v>
@@ -2348,7 +2348,7 @@
         <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>160.705</v>
+        <v>295.005</v>
       </c>
       <c r="J7" s="1">
         <v>3000</v>
@@ -2575,7 +2575,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="1">
-        <v>15011</v>
+        <v>30000</v>
       </c>
       <c r="G8" s="1">
         <v>1</v>
@@ -2584,7 +2584,7 @@
         <v>0</v>
       </c>
       <c r="I8" s="1">
-        <v>161.406</v>
+        <v>296.805</v>
       </c>
       <c r="J8" s="1">
         <v>3000</v>
@@ -2811,7 +2811,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="1">
-        <v>15007</v>
+        <v>30008</v>
       </c>
       <c r="G9" s="1">
         <v>1</v>
@@ -2820,7 +2820,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>161.406</v>
+        <v>297.205</v>
       </c>
       <c r="J9" s="1">
         <v>3000</v>
@@ -3047,7 +3047,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="1">
-        <v>15007</v>
+        <v>30009</v>
       </c>
       <c r="G10" s="1">
         <v>1</v>
@@ -3056,7 +3056,7 @@
         <v>0</v>
       </c>
       <c r="I10" s="1">
-        <v>162.005</v>
+        <v>297.006</v>
       </c>
       <c r="J10" s="1">
         <v>3000</v>
@@ -3283,7 +3283,7 @@
         <v>0</v>
       </c>
       <c r="F11" s="1">
-        <v>15007</v>
+        <v>30001</v>
       </c>
       <c r="G11" s="1">
         <v>1</v>
@@ -3292,7 +3292,7 @@
         <v>0</v>
       </c>
       <c r="I11" s="1">
-        <v>161.806</v>
+        <v>297.805</v>
       </c>
       <c r="J11" s="1">
         <v>3000</v>
@@ -3519,7 +3519,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="1">
-        <v>15004</v>
+        <v>30000</v>
       </c>
       <c r="G12" s="1">
         <v>1</v>
@@ -3528,7 +3528,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="1">
-        <v>156.339</v>
+        <v>297.505</v>
       </c>
       <c r="J12" s="1">
         <v>3000</v>
@@ -3755,7 +3755,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="1">
-        <v>15007</v>
+        <v>30007</v>
       </c>
       <c r="G13" s="1">
         <v>1</v>
@@ -3764,7 +3764,7 @@
         <v>0</v>
       </c>
       <c r="I13" s="1">
-        <v>162.106</v>
+        <v>299.704</v>
       </c>
       <c r="J13" s="1">
         <v>3000</v>
@@ -3991,7 +3991,7 @@
         <v>0</v>
       </c>
       <c r="F14" s="1">
-        <v>15007</v>
+        <v>30005</v>
       </c>
       <c r="G14" s="1">
         <v>1</v>
@@ -4000,7 +4000,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="1">
-        <v>161.706</v>
+        <v>299.304</v>
       </c>
       <c r="J14" s="1">
         <v>3000</v>
@@ -4227,7 +4227,7 @@
         <v>0</v>
       </c>
       <c r="F15" s="1">
-        <v>15008</v>
+        <v>30005</v>
       </c>
       <c r="G15" s="1">
         <v>1</v>
@@ -4236,7 +4236,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="1">
-        <v>160.805</v>
+        <v>296.805</v>
       </c>
       <c r="J15" s="1">
         <v>3000</v>
@@ -4463,7 +4463,7 @@
         <v>0</v>
       </c>
       <c r="F16" s="1">
-        <v>15007</v>
+        <v>30007</v>
       </c>
       <c r="G16" s="1">
         <v>1</v>
@@ -4472,7 +4472,7 @@
         <v>0</v>
       </c>
       <c r="I16" s="1">
-        <v>162.205</v>
+        <v>298.904</v>
       </c>
       <c r="J16" s="1">
         <v>3000</v>
@@ -4699,7 +4699,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="1">
-        <v>15004</v>
+        <v>30009</v>
       </c>
       <c r="G17" s="1">
         <v>1</v>
@@ -4708,7 +4708,7 @@
         <v>0</v>
       </c>
       <c r="I17" s="1">
-        <v>161.106</v>
+        <v>297.906</v>
       </c>
       <c r="J17" s="1">
         <v>3000</v>
@@ -4935,7 +4935,7 @@
         <v>0</v>
       </c>
       <c r="F18" s="1">
-        <v>15004</v>
+        <v>30002</v>
       </c>
       <c r="G18" s="1">
         <v>1</v>
@@ -4944,7 +4944,7 @@
         <v>0</v>
       </c>
       <c r="I18" s="1">
-        <v>161.906</v>
+        <v>300.005</v>
       </c>
       <c r="J18" s="1">
         <v>3000</v>
@@ -5171,7 +5171,7 @@
         <v>0</v>
       </c>
       <c r="F19" s="1">
-        <v>15002</v>
+        <v>30001</v>
       </c>
       <c r="G19" s="1">
         <v>1</v>
@@ -5180,7 +5180,7 @@
         <v>0</v>
       </c>
       <c r="I19" s="1">
-        <v>161.606</v>
+        <v>300.005</v>
       </c>
       <c r="J19" s="1">
         <v>3000</v>
@@ -5407,7 +5407,7 @@
         <v>0</v>
       </c>
       <c r="F20" s="1">
-        <v>15003</v>
+        <v>30002</v>
       </c>
       <c r="G20" s="1">
         <v>1</v>
@@ -5416,7 +5416,7 @@
         <v>0</v>
       </c>
       <c r="I20" s="1">
-        <v>161.906</v>
+        <v>298.005</v>
       </c>
       <c r="J20" s="1">
         <v>3000</v>
@@ -5643,7 +5643,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="1">
-        <v>15004</v>
+        <v>30001</v>
       </c>
       <c r="G21" s="1">
         <v>1</v>
@@ -5652,7 +5652,7 @@
         <v>0</v>
       </c>
       <c r="I21" s="1">
-        <v>161.806</v>
+        <v>299.805</v>
       </c>
       <c r="J21" s="1">
         <v>3000</v>
@@ -5879,7 +5879,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="1">
-        <v>15004</v>
+        <v>30002</v>
       </c>
       <c r="G22" s="1">
         <v>1</v>
@@ -5888,7 +5888,7 @@
         <v>0</v>
       </c>
       <c r="I22" s="1">
-        <v>162.206</v>
+        <v>297.104</v>
       </c>
       <c r="J22" s="1">
         <v>3000</v>
@@ -6115,7 +6115,7 @@
         <v>0</v>
       </c>
       <c r="F23" s="1">
-        <v>15001</v>
+        <v>30007</v>
       </c>
       <c r="G23" s="1">
         <v>1</v>
@@ -6124,7 +6124,7 @@
         <v>0</v>
       </c>
       <c r="I23" s="1">
-        <v>163.106</v>
+        <v>301.905</v>
       </c>
       <c r="J23" s="1">
         <v>3000</v>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="F24" s="1">
-        <v>15009</v>
+        <v>30001</v>
       </c>
       <c r="G24" s="1">
         <v>1</v>
@@ -6360,7 +6360,7 @@
         <v>0</v>
       </c>
       <c r="I24" s="1">
-        <v>162.506</v>
+        <v>305.405</v>
       </c>
       <c r="J24" s="1">
         <v>3000</v>
@@ -6587,7 +6587,7 @@
         <v>0</v>
       </c>
       <c r="F25" s="1">
-        <v>15000</v>
+        <v>30007</v>
       </c>
       <c r="G25" s="1">
         <v>1</v>
@@ -6596,7 +6596,7 @@
         <v>0</v>
       </c>
       <c r="I25" s="1">
-        <v>163.606</v>
+        <v>304.505</v>
       </c>
       <c r="J25" s="1">
         <v>3000</v>
@@ -6823,7 +6823,7 @@
         <v>0</v>
       </c>
       <c r="F26" s="1">
-        <v>15006</v>
+        <v>30000</v>
       </c>
       <c r="G26" s="1">
         <v>1</v>
@@ -6832,7 +6832,7 @@
         <v>0</v>
       </c>
       <c r="I26" s="1">
-        <v>161.806</v>
+        <v>301.705</v>
       </c>
       <c r="J26" s="1">
         <v>3000</v>
@@ -7059,7 +7059,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="1">
-        <v>15001</v>
+        <v>30006</v>
       </c>
       <c r="G27" s="1">
         <v>1</v>
@@ -7068,7 +7068,7 @@
         <v>0</v>
       </c>
       <c r="I27" s="1">
-        <v>162.905</v>
+        <v>302.505</v>
       </c>
       <c r="J27" s="1">
         <v>3000</v>
@@ -7295,7 +7295,7 @@
         <v>0</v>
       </c>
       <c r="F28" s="1">
-        <v>15002</v>
+        <v>30005</v>
       </c>
       <c r="G28" s="1">
         <v>1</v>
@@ -7304,7 +7304,7 @@
         <v>0</v>
       </c>
       <c r="I28" s="1">
-        <v>162.806</v>
+        <v>302.404</v>
       </c>
       <c r="J28" s="1">
         <v>3000</v>
@@ -7531,7 +7531,7 @@
         <v>0</v>
       </c>
       <c r="F29" s="1">
-        <v>15005</v>
+        <v>30008</v>
       </c>
       <c r="G29" s="1">
         <v>1</v>
@@ -7540,7 +7540,7 @@
         <v>0</v>
       </c>
       <c r="I29" s="1">
-        <v>163.006</v>
+        <v>304.105</v>
       </c>
       <c r="J29" s="1">
         <v>3000</v>
@@ -7767,7 +7767,7 @@
         <v>0</v>
       </c>
       <c r="F30" s="1">
-        <v>15002</v>
+        <v>30006</v>
       </c>
       <c r="G30" s="1">
         <v>1</v>
@@ -7776,7 +7776,7 @@
         <v>0</v>
       </c>
       <c r="I30" s="1">
-        <v>162.906</v>
+        <v>302.705</v>
       </c>
       <c r="J30" s="1">
         <v>3000</v>
@@ -8003,7 +8003,7 @@
         <v>0</v>
       </c>
       <c r="F31" s="1">
-        <v>15002</v>
+        <v>30009</v>
       </c>
       <c r="G31" s="1">
         <v>1</v>
@@ -8012,7 +8012,7 @@
         <v>0</v>
       </c>
       <c r="I31" s="1">
-        <v>162.406</v>
+        <v>303.405</v>
       </c>
       <c r="J31" s="1">
         <v>3000</v>
@@ -8239,7 +8239,7 @@
         <v>0</v>
       </c>
       <c r="F32" s="1">
-        <v>15003</v>
+        <v>30002</v>
       </c>
       <c r="G32" s="1">
         <v>1</v>
@@ -8248,7 +8248,7 @@
         <v>0</v>
       </c>
       <c r="I32" s="1">
-        <v>162.006</v>
+        <v>300.105</v>
       </c>
       <c r="J32" s="1">
         <v>3000</v>

</xml_diff>